<commit_message>
Clarify which service page sections duplicate the homepage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGAbrQV8r5PoLynyqeZRVA
</commit_message>
<xml_diff>
--- a/orbitalx-seo-audit.xlsx
+++ b/orbitalx-seo-audit.xlsx
@@ -596,13 +596,13 @@
     <t xml:space="preserve">Service pages duplicate the homepage</t>
   </si>
   <si>
-    <t xml:space="preserve">46–63% of each main service page's text is copied from the homepage.</t>
+    <t xml:space="preserve">46–63% of each main service page's text is copied from the homepage. Identical sections: proof bar, 'One system that runs your entire pipeline engine', 'How it works', 'What it costs to build this yourself', testimonials, 'See how your target accounts see you'. Partly copied: 'Real results' and FAQs.</t>
   </si>
   <si>
     <t xml:space="preserve">Thin / duplicate signals</t>
   </si>
   <si>
-    <t xml:space="preserve">Rewrite the 'broken', 'how it works' and FAQ blocks per service.</t>
+    <t xml:space="preserve">Rewrite 'One system…', 'How it works' and 'What it costs…' per service; make FAQs and results service-specific. Keep proof bar and testimonials.</t>
   </si>
   <si>
     <t xml:space="preserve">G16</t>
@@ -5600,11 +5600,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="4013204"/>
-        <c:axId val="72198085"/>
+        <c:axId val="85169958"/>
+        <c:axId val="36620475"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="4013204"/>
+        <c:axId val="85169958"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5636,7 +5636,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72198085"/>
+        <c:crossAx val="36620475"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5644,7 +5644,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="72198085"/>
+        <c:axId val="36620475"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5686,7 +5686,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4013204"/>
+        <c:crossAx val="85169958"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6390,11 +6390,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="64017951"/>
-        <c:axId val="38289114"/>
+        <c:axId val="51679653"/>
+        <c:axId val="30840619"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="64017951"/>
+        <c:axId val="51679653"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6426,7 +6426,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38289114"/>
+        <c:crossAx val="30840619"/>
         <c:crosses val="max"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6434,7 +6434,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="38289114"/>
+        <c:axId val="30840619"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -6476,7 +6476,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64017951"/>
+        <c:crossAx val="51679653"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -21766,7 +21766,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
         <v>172</v>
       </c>
@@ -28216,7 +28216,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{962C4853-8B60-4840-A255-EBB64DA4FE72}</x14:id>
+          <x14:id>{D197C9BE-FAAE-4950-A832-B6ECE22FACCC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -28234,7 +28234,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{962C4853-8B60-4840-A255-EBB64DA4FE72}">
+          <x14:cfRule type="dataBar" id="{D197C9BE-FAAE-4950-A832-B6ECE22FACCC}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>